<commit_message>
Actualización definitiva de tareas.xlsx
</commit_message>
<xml_diff>
--- a/tareas.xlsx
+++ b/tareas.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="810" uniqueCount="106">
   <si>
     <t>Etapa</t>
   </si>
@@ -240,6 +240,9 @@
   </si>
   <si>
     <t>RNOF Perfil Cliente</t>
+  </si>
+  <si>
+    <t>Automatizacion de Reportes al Cliente</t>
   </si>
   <si>
     <t>RNOF Perfil Director</t>
@@ -2592,28 +2595,28 @@
     </row>
     <row r="43" ht="29.25" customHeight="1">
       <c r="A43" s="10" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>58</v>
+        <v>21</v>
       </c>
       <c r="C43" s="12" t="s">
         <v>76</v>
       </c>
       <c r="D43" s="13" t="s">
-        <v>74</v>
+        <v>15</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>69</v>
+        <v>16</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="G43" s="14">
-        <v>46288.0</v>
+        <v>46285.0</v>
       </c>
       <c r="H43" s="14">
-        <v>46289.0</v>
+        <v>46285.0</v>
       </c>
       <c r="I43" s="14"/>
       <c r="J43" s="15"/>
@@ -2640,513 +2643,532 @@
       <c r="AE43" s="16"/>
     </row>
     <row r="44" ht="29.25" customHeight="1">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="10" t="s">
         <v>26</v>
       </c>
       <c r="B44" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C44" s="22" t="s">
+      <c r="C44" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="D44" s="7" t="s">
+      <c r="D44" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="E44" s="7"/>
-      <c r="F44" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G44" s="8">
+      <c r="E44" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F44" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G44" s="14">
         <v>46288.0</v>
       </c>
-      <c r="H44" s="8">
+      <c r="H44" s="14">
         <v>46289.0</v>
       </c>
-      <c r="I44" s="8"/>
-      <c r="J44" s="17"/>
-      <c r="K44" s="9"/>
-      <c r="L44" s="9"/>
+      <c r="I44" s="14"/>
+      <c r="J44" s="15"/>
+      <c r="K44" s="15"/>
+      <c r="L44" s="15"/>
+      <c r="M44" s="16"/>
+      <c r="N44" s="16"/>
+      <c r="O44" s="16"/>
+      <c r="P44" s="16"/>
+      <c r="Q44" s="16"/>
+      <c r="R44" s="16"/>
+      <c r="S44" s="16"/>
+      <c r="T44" s="16"/>
+      <c r="U44" s="16"/>
+      <c r="V44" s="16"/>
+      <c r="W44" s="16"/>
+      <c r="X44" s="16"/>
+      <c r="Y44" s="16"/>
+      <c r="Z44" s="16"/>
+      <c r="AA44" s="16"/>
+      <c r="AB44" s="16"/>
+      <c r="AC44" s="16"/>
+      <c r="AD44" s="16"/>
+      <c r="AE44" s="16"/>
     </row>
     <row r="45" ht="29.25" customHeight="1">
-      <c r="A45" s="10" t="s">
+      <c r="A45" s="4" t="s">
         <v>26</v>
       </c>
       <c r="B45" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C45" s="12" t="s">
+      <c r="C45" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="D45" s="13" t="s">
+      <c r="D45" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E45" s="13"/>
-      <c r="F45" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="G45" s="14">
-        <v>46285.0</v>
-      </c>
-      <c r="H45" s="14">
+      <c r="E45" s="7"/>
+      <c r="F45" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G45" s="8">
+        <v>46288.0</v>
+      </c>
+      <c r="H45" s="8">
         <v>46289.0</v>
       </c>
-      <c r="I45" s="14"/>
-      <c r="J45" s="15"/>
-      <c r="K45" s="15"/>
-      <c r="L45" s="15"/>
-      <c r="M45" s="16"/>
-      <c r="N45" s="16"/>
-      <c r="O45" s="16"/>
-      <c r="P45" s="16"/>
-      <c r="Q45" s="16"/>
-      <c r="R45" s="16"/>
-      <c r="S45" s="16"/>
-      <c r="T45" s="16"/>
-      <c r="U45" s="16"/>
-      <c r="V45" s="16"/>
-      <c r="W45" s="16"/>
-      <c r="X45" s="16"/>
-      <c r="Y45" s="16"/>
-      <c r="Z45" s="16"/>
-      <c r="AA45" s="16"/>
-      <c r="AB45" s="16"/>
-      <c r="AC45" s="16"/>
-      <c r="AD45" s="16"/>
-      <c r="AE45" s="16"/>
+      <c r="I45" s="8"/>
+      <c r="J45" s="17"/>
+      <c r="K45" s="9"/>
+      <c r="L45" s="9"/>
     </row>
     <row r="46" ht="29.25" customHeight="1">
-      <c r="A46" s="4" t="s">
+      <c r="A46" s="10" t="s">
         <v>26</v>
       </c>
       <c r="B46" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C46" s="22" t="s">
+      <c r="C46" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="D46" s="7" t="s">
+      <c r="D46" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="E46" s="7"/>
-      <c r="F46" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G46" s="8">
-        <v>46286.0</v>
-      </c>
-      <c r="H46" s="8">
-        <v>46288.0</v>
-      </c>
-      <c r="I46" s="8"/>
-      <c r="J46" s="17"/>
-      <c r="K46" s="9"/>
-      <c r="L46" s="9"/>
+      <c r="E46" s="13"/>
+      <c r="F46" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="G46" s="14">
+        <v>46285.0</v>
+      </c>
+      <c r="H46" s="14">
+        <v>46289.0</v>
+      </c>
+      <c r="I46" s="14"/>
+      <c r="J46" s="15"/>
+      <c r="K46" s="15"/>
+      <c r="L46" s="15"/>
+      <c r="M46" s="16"/>
+      <c r="N46" s="16"/>
+      <c r="O46" s="16"/>
+      <c r="P46" s="16"/>
+      <c r="Q46" s="16"/>
+      <c r="R46" s="16"/>
+      <c r="S46" s="16"/>
+      <c r="T46" s="16"/>
+      <c r="U46" s="16"/>
+      <c r="V46" s="16"/>
+      <c r="W46" s="16"/>
+      <c r="X46" s="16"/>
+      <c r="Y46" s="16"/>
+      <c r="Z46" s="16"/>
+      <c r="AA46" s="16"/>
+      <c r="AB46" s="16"/>
+      <c r="AC46" s="16"/>
+      <c r="AD46" s="16"/>
+      <c r="AE46" s="16"/>
     </row>
     <row r="47" ht="29.25" customHeight="1">
-      <c r="A47" s="10" t="s">
+      <c r="A47" s="4" t="s">
         <v>26</v>
       </c>
       <c r="B47" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C47" s="12" t="s">
+      <c r="C47" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="D47" s="13" t="s">
+      <c r="D47" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E47" s="13"/>
-      <c r="F47" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="G47" s="14">
+      <c r="E47" s="7"/>
+      <c r="F47" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G47" s="8">
         <v>46286.0</v>
       </c>
-      <c r="H47" s="14">
+      <c r="H47" s="8">
         <v>46288.0</v>
       </c>
-      <c r="I47" s="14"/>
-      <c r="J47" s="15"/>
-      <c r="K47" s="15"/>
-      <c r="L47" s="15"/>
-      <c r="M47" s="16"/>
-      <c r="N47" s="16"/>
-      <c r="O47" s="16"/>
-      <c r="P47" s="16"/>
-      <c r="Q47" s="16"/>
-      <c r="R47" s="16"/>
-      <c r="S47" s="16"/>
-      <c r="T47" s="16"/>
-      <c r="U47" s="16"/>
-      <c r="V47" s="16"/>
-      <c r="W47" s="16"/>
-      <c r="X47" s="16"/>
-      <c r="Y47" s="16"/>
-      <c r="Z47" s="16"/>
-      <c r="AA47" s="16"/>
-      <c r="AB47" s="16"/>
-      <c r="AC47" s="16"/>
-      <c r="AD47" s="16"/>
-      <c r="AE47" s="16"/>
+      <c r="I47" s="8"/>
+      <c r="J47" s="17"/>
+      <c r="K47" s="9"/>
+      <c r="L47" s="9"/>
     </row>
     <row r="48" ht="29.25" customHeight="1">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="10" t="s">
         <v>26</v>
       </c>
       <c r="B48" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="C48" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="D48" s="7" t="s">
+      <c r="C48" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D48" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="E48" s="7"/>
-      <c r="F48" s="7"/>
-      <c r="G48" s="8">
+      <c r="E48" s="13"/>
+      <c r="F48" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G48" s="14">
         <v>46286.0</v>
       </c>
-      <c r="H48" s="8">
+      <c r="H48" s="14">
         <v>46288.0</v>
       </c>
-      <c r="I48" s="8"/>
-      <c r="J48" s="17"/>
-      <c r="K48" s="9"/>
-      <c r="L48" s="9"/>
+      <c r="I48" s="14"/>
+      <c r="J48" s="15"/>
+      <c r="K48" s="15"/>
+      <c r="L48" s="15"/>
+      <c r="M48" s="16"/>
+      <c r="N48" s="16"/>
+      <c r="O48" s="16"/>
+      <c r="P48" s="16"/>
+      <c r="Q48" s="16"/>
+      <c r="R48" s="16"/>
+      <c r="S48" s="16"/>
+      <c r="T48" s="16"/>
+      <c r="U48" s="16"/>
+      <c r="V48" s="16"/>
+      <c r="W48" s="16"/>
+      <c r="X48" s="16"/>
+      <c r="Y48" s="16"/>
+      <c r="Z48" s="16"/>
+      <c r="AA48" s="16"/>
+      <c r="AB48" s="16"/>
+      <c r="AC48" s="16"/>
+      <c r="AD48" s="16"/>
+      <c r="AE48" s="16"/>
     </row>
     <row r="49" ht="29.25" customHeight="1">
-      <c r="A49" s="10" t="s">
+      <c r="A49" s="4" t="s">
         <v>26</v>
       </c>
       <c r="B49" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="C49" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="8">
+        <v>46286.0</v>
+      </c>
+      <c r="H49" s="8">
+        <v>46288.0</v>
+      </c>
+      <c r="I49" s="8"/>
+      <c r="J49" s="17"/>
+      <c r="K49" s="9"/>
+      <c r="L49" s="9"/>
+    </row>
+    <row r="50" ht="29.25" customHeight="1">
+      <c r="A50" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B50" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="D49" s="13" t="s">
+      <c r="C50" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="D50" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="E49" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="F49" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="G49" s="14">
+      <c r="E50" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F50" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G50" s="14">
         <v>46287.0</v>
       </c>
-      <c r="H49" s="14">
+      <c r="H50" s="14">
         <v>46290.0</v>
       </c>
-      <c r="I49" s="14"/>
-      <c r="J49" s="15"/>
-      <c r="K49" s="15"/>
-      <c r="L49" s="15"/>
-      <c r="M49" s="16"/>
-      <c r="N49" s="16"/>
-      <c r="O49" s="16"/>
-      <c r="P49" s="16"/>
-      <c r="Q49" s="16"/>
-      <c r="R49" s="16"/>
-      <c r="S49" s="16"/>
-      <c r="T49" s="16"/>
-      <c r="U49" s="16"/>
-      <c r="V49" s="16"/>
-      <c r="W49" s="16"/>
-      <c r="X49" s="16"/>
-      <c r="Y49" s="16"/>
-      <c r="Z49" s="16"/>
-      <c r="AA49" s="16"/>
-      <c r="AB49" s="16"/>
-      <c r="AC49" s="16"/>
-      <c r="AD49" s="16"/>
-      <c r="AE49" s="16"/>
-    </row>
-    <row r="50" ht="29.25" customHeight="1">
-      <c r="A50" s="4" t="s">
+      <c r="I50" s="14"/>
+      <c r="J50" s="15"/>
+      <c r="K50" s="15"/>
+      <c r="L50" s="15"/>
+      <c r="M50" s="16"/>
+      <c r="N50" s="16"/>
+      <c r="O50" s="16"/>
+      <c r="P50" s="16"/>
+      <c r="Q50" s="16"/>
+      <c r="R50" s="16"/>
+      <c r="S50" s="16"/>
+      <c r="T50" s="16"/>
+      <c r="U50" s="16"/>
+      <c r="V50" s="16"/>
+      <c r="W50" s="16"/>
+      <c r="X50" s="16"/>
+      <c r="Y50" s="16"/>
+      <c r="Z50" s="16"/>
+      <c r="AA50" s="16"/>
+      <c r="AB50" s="16"/>
+      <c r="AC50" s="16"/>
+      <c r="AD50" s="16"/>
+      <c r="AE50" s="16"/>
+    </row>
+    <row r="51" ht="29.25" customHeight="1">
+      <c r="A51" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B50" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D50" s="7" t="s">
+      <c r="B51" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="D51" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E50" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="F50" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="G50" s="8">
+      <c r="E51" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G51" s="8">
         <v>46288.0</v>
       </c>
-      <c r="H50" s="8">
+      <c r="H51" s="8">
         <v>46290.0</v>
       </c>
-      <c r="I50" s="8"/>
-      <c r="J50" s="17"/>
-      <c r="K50" s="9"/>
-      <c r="L50" s="9"/>
-    </row>
-    <row r="51" ht="29.25" customHeight="1">
-      <c r="A51" s="10" t="s">
+      <c r="I51" s="8"/>
+      <c r="J51" s="17"/>
+      <c r="K51" s="9"/>
+      <c r="L51" s="9"/>
+    </row>
+    <row r="52" ht="29.25" customHeight="1">
+      <c r="A52" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B51" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="C51" s="12" t="s">
+      <c r="B52" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="D51" s="13" t="s">
+      <c r="C52" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="D52" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="E51" s="13"/>
-      <c r="F51" s="13" t="s">
+      <c r="E52" s="13"/>
+      <c r="F52" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="G51" s="14">
+      <c r="G52" s="14">
         <v>46291.0</v>
       </c>
-      <c r="H51" s="14">
+      <c r="H52" s="14">
         <v>46291.0</v>
       </c>
-      <c r="I51" s="14"/>
-      <c r="J51" s="15"/>
-      <c r="K51" s="15"/>
-      <c r="L51" s="15"/>
-      <c r="M51" s="16"/>
-      <c r="N51" s="16"/>
-      <c r="O51" s="16"/>
-      <c r="P51" s="16"/>
-      <c r="Q51" s="16"/>
-      <c r="R51" s="16"/>
-      <c r="S51" s="16"/>
-      <c r="T51" s="16"/>
-      <c r="U51" s="16"/>
-      <c r="V51" s="16"/>
-      <c r="W51" s="16"/>
-      <c r="X51" s="16"/>
-      <c r="Y51" s="16"/>
-      <c r="Z51" s="16"/>
-      <c r="AA51" s="16"/>
-      <c r="AB51" s="16"/>
-      <c r="AC51" s="16"/>
-      <c r="AD51" s="16"/>
-      <c r="AE51" s="16"/>
-    </row>
-    <row r="52" ht="29.25" customHeight="1">
-      <c r="A52" s="4" t="s">
+      <c r="I52" s="14"/>
+      <c r="J52" s="15"/>
+      <c r="K52" s="15"/>
+      <c r="L52" s="15"/>
+      <c r="M52" s="16"/>
+      <c r="N52" s="16"/>
+      <c r="O52" s="16"/>
+      <c r="P52" s="16"/>
+      <c r="Q52" s="16"/>
+      <c r="R52" s="16"/>
+      <c r="S52" s="16"/>
+      <c r="T52" s="16"/>
+      <c r="U52" s="16"/>
+      <c r="V52" s="16"/>
+      <c r="W52" s="16"/>
+      <c r="X52" s="16"/>
+      <c r="Y52" s="16"/>
+      <c r="Z52" s="16"/>
+      <c r="AA52" s="16"/>
+      <c r="AB52" s="16"/>
+      <c r="AC52" s="16"/>
+      <c r="AD52" s="16"/>
+      <c r="AE52" s="16"/>
+    </row>
+    <row r="53" ht="29.25" customHeight="1">
+      <c r="A53" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B52" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C52" s="6" t="s">
+      <c r="B53" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D52" s="7" t="s">
+      <c r="C53" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D53" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E52" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="F52" s="7" t="s">
+      <c r="E53" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F53" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="G52" s="8">
+      <c r="G53" s="8">
         <v>46291.0</v>
       </c>
-      <c r="H52" s="8">
+      <c r="H53" s="8">
         <v>46291.0</v>
       </c>
-      <c r="I52" s="8"/>
-      <c r="J52" s="9"/>
-      <c r="K52" s="9"/>
-      <c r="L52" s="9"/>
-    </row>
-    <row r="53" ht="29.25" customHeight="1">
-      <c r="A53" s="10" t="s">
+      <c r="I53" s="8"/>
+      <c r="J53" s="9"/>
+      <c r="K53" s="9"/>
+      <c r="L53" s="9"/>
+    </row>
+    <row r="54" ht="29.25" customHeight="1">
+      <c r="A54" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B53" s="11" t="s">
-        <v>86</v>
-      </c>
-      <c r="C53" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="D53" s="13" t="s">
+      <c r="B54" s="11" t="s">
+        <v>87</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D54" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="E53" s="13"/>
-      <c r="F53" s="13" t="s">
+      <c r="E54" s="13"/>
+      <c r="F54" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="G53" s="14">
+      <c r="G54" s="14">
         <v>46291.0</v>
       </c>
-      <c r="H53" s="14">
+      <c r="H54" s="14">
         <v>46291.0</v>
       </c>
-      <c r="I53" s="14"/>
-      <c r="J53" s="15"/>
-      <c r="K53" s="15"/>
-      <c r="L53" s="15"/>
-      <c r="M53" s="16"/>
-      <c r="N53" s="16"/>
-      <c r="O53" s="16"/>
-      <c r="P53" s="16"/>
-      <c r="Q53" s="16"/>
-      <c r="R53" s="16"/>
-      <c r="S53" s="16"/>
-      <c r="T53" s="16"/>
-      <c r="U53" s="16"/>
-      <c r="V53" s="16"/>
-      <c r="W53" s="16"/>
-      <c r="X53" s="16"/>
-      <c r="Y53" s="16"/>
-      <c r="Z53" s="16"/>
-      <c r="AA53" s="16"/>
-      <c r="AB53" s="16"/>
-      <c r="AC53" s="16"/>
-      <c r="AD53" s="16"/>
-      <c r="AE53" s="16"/>
-    </row>
-    <row r="54" ht="29.25" customHeight="1">
-      <c r="A54" s="4" t="s">
+      <c r="I54" s="14"/>
+      <c r="J54" s="15"/>
+      <c r="K54" s="15"/>
+      <c r="L54" s="15"/>
+      <c r="M54" s="16"/>
+      <c r="N54" s="16"/>
+      <c r="O54" s="16"/>
+      <c r="P54" s="16"/>
+      <c r="Q54" s="16"/>
+      <c r="R54" s="16"/>
+      <c r="S54" s="16"/>
+      <c r="T54" s="16"/>
+      <c r="U54" s="16"/>
+      <c r="V54" s="16"/>
+      <c r="W54" s="16"/>
+      <c r="X54" s="16"/>
+      <c r="Y54" s="16"/>
+      <c r="Z54" s="16"/>
+      <c r="AA54" s="16"/>
+      <c r="AB54" s="16"/>
+      <c r="AC54" s="16"/>
+      <c r="AD54" s="16"/>
+      <c r="AE54" s="16"/>
+    </row>
+    <row r="55" ht="29.25" customHeight="1">
+      <c r="A55" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B54" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="D54" s="7" t="s">
+      <c r="B55" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D55" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E54" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="F54" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="G54" s="8">
+      <c r="E55" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G55" s="8">
         <v>46286.0</v>
       </c>
-      <c r="H54" s="8">
+      <c r="H55" s="8">
         <v>46293.0</v>
       </c>
-      <c r="I54" s="8"/>
-      <c r="J54" s="9"/>
-      <c r="K54" s="9"/>
-      <c r="L54" s="9"/>
-    </row>
-    <row r="55" ht="29.25" customHeight="1">
-      <c r="A55" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B55" s="11" t="s">
+      <c r="I55" s="8"/>
+      <c r="J55" s="9"/>
+      <c r="K55" s="9"/>
+      <c r="L55" s="9"/>
+    </row>
+    <row r="56" ht="29.25" customHeight="1">
+      <c r="A56" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="C55" s="12" t="s">
+      <c r="B56" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="D55" s="13" t="s">
+      <c r="C56" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="D56" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="E55" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="F55" s="13" t="s">
+      <c r="E56" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F56" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="G55" s="14">
+      <c r="G56" s="14">
         <v>46289.0</v>
       </c>
-      <c r="H55" s="14">
+      <c r="H56" s="14">
         <v>46289.0</v>
       </c>
-      <c r="I55" s="14"/>
-      <c r="J55" s="15"/>
-      <c r="K55" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="L55" s="15"/>
-      <c r="M55" s="16"/>
-      <c r="N55" s="16"/>
-      <c r="O55" s="16"/>
-      <c r="P55" s="16"/>
-      <c r="Q55" s="16"/>
-      <c r="R55" s="16"/>
-      <c r="S55" s="16"/>
-      <c r="T55" s="16"/>
-      <c r="U55" s="16"/>
-      <c r="V55" s="16"/>
-      <c r="W55" s="16"/>
-      <c r="X55" s="16"/>
-      <c r="Y55" s="16"/>
-      <c r="Z55" s="16"/>
-      <c r="AA55" s="16"/>
-      <c r="AB55" s="16"/>
-      <c r="AC55" s="16"/>
-      <c r="AD55" s="16"/>
-      <c r="AE55" s="16"/>
-    </row>
-    <row r="56" ht="29.25" customHeight="1">
-      <c r="A56" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B56" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="E56" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="F56" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="G56" s="8">
-        <v>46289.0</v>
-      </c>
-      <c r="H56" s="8">
-        <v>46289.0</v>
-      </c>
-      <c r="I56" s="8"/>
-      <c r="J56" s="9"/>
-      <c r="K56" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="L56" s="9"/>
+      <c r="I56" s="14"/>
+      <c r="J56" s="15"/>
+      <c r="K56" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="L56" s="15"/>
+      <c r="M56" s="16"/>
+      <c r="N56" s="16"/>
+      <c r="O56" s="16"/>
+      <c r="P56" s="16"/>
+      <c r="Q56" s="16"/>
+      <c r="R56" s="16"/>
+      <c r="S56" s="16"/>
+      <c r="T56" s="16"/>
+      <c r="U56" s="16"/>
+      <c r="V56" s="16"/>
+      <c r="W56" s="16"/>
+      <c r="X56" s="16"/>
+      <c r="Y56" s="16"/>
+      <c r="Z56" s="16"/>
+      <c r="AA56" s="16"/>
+      <c r="AB56" s="16"/>
+      <c r="AC56" s="16"/>
+      <c r="AD56" s="16"/>
+      <c r="AE56" s="16"/>
     </row>
     <row r="57" ht="29.25" customHeight="1">
       <c r="A57" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B57" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D57" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E57" s="7"/>
+      <c r="E57" s="7" t="s">
+        <v>69</v>
+      </c>
       <c r="F57" s="7" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="G57" s="8">
         <v>46289.0</v>
@@ -3156,249 +3178,263 @@
       </c>
       <c r="I57" s="8"/>
       <c r="J57" s="9"/>
-      <c r="K57" s="9"/>
+      <c r="K57" s="9" t="s">
+        <v>94</v>
+      </c>
       <c r="L57" s="9"/>
     </row>
     <row r="58" ht="29.25" customHeight="1">
-      <c r="A58" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B58" s="11" t="s">
+      <c r="A58" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C58" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C58" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="D58" s="13" t="s">
+      <c r="D58" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E58" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="F58" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="G58" s="14">
+      <c r="E58" s="7"/>
+      <c r="F58" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G58" s="8">
+        <v>46289.0</v>
+      </c>
+      <c r="H58" s="8">
+        <v>46289.0</v>
+      </c>
+      <c r="I58" s="8"/>
+      <c r="J58" s="9"/>
+      <c r="K58" s="9"/>
+      <c r="L58" s="9"/>
+    </row>
+    <row r="59" ht="29.25" customHeight="1">
+      <c r="A59" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B59" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="C59" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="D59" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="E59" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F59" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G59" s="14">
         <v>46286.0</v>
       </c>
-      <c r="H58" s="14">
+      <c r="H59" s="14">
         <v>46293.0</v>
       </c>
-      <c r="I58" s="14"/>
-      <c r="J58" s="15"/>
-      <c r="K58" s="15"/>
-      <c r="L58" s="15"/>
-      <c r="M58" s="16"/>
-      <c r="N58" s="16"/>
-      <c r="O58" s="16"/>
-      <c r="P58" s="16"/>
-      <c r="Q58" s="16"/>
-      <c r="R58" s="16"/>
-      <c r="S58" s="16"/>
-      <c r="T58" s="16"/>
-      <c r="U58" s="16"/>
-      <c r="V58" s="16"/>
-      <c r="W58" s="16"/>
-      <c r="X58" s="16"/>
-      <c r="Y58" s="16"/>
-      <c r="Z58" s="16"/>
-      <c r="AA58" s="16"/>
-      <c r="AB58" s="16"/>
-      <c r="AC58" s="16"/>
-      <c r="AD58" s="16"/>
-      <c r="AE58" s="16"/>
-    </row>
-    <row r="59" ht="29.25" customHeight="1">
-      <c r="A59" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B59" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="D59" s="7" t="s">
+      <c r="I59" s="14"/>
+      <c r="J59" s="15"/>
+      <c r="K59" s="15"/>
+      <c r="L59" s="15"/>
+      <c r="M59" s="16"/>
+      <c r="N59" s="16"/>
+      <c r="O59" s="16"/>
+      <c r="P59" s="16"/>
+      <c r="Q59" s="16"/>
+      <c r="R59" s="16"/>
+      <c r="S59" s="16"/>
+      <c r="T59" s="16"/>
+      <c r="U59" s="16"/>
+      <c r="V59" s="16"/>
+      <c r="W59" s="16"/>
+      <c r="X59" s="16"/>
+      <c r="Y59" s="16"/>
+      <c r="Z59" s="16"/>
+      <c r="AA59" s="16"/>
+      <c r="AB59" s="16"/>
+      <c r="AC59" s="16"/>
+      <c r="AD59" s="16"/>
+      <c r="AE59" s="16"/>
+    </row>
+    <row r="60" ht="29.25" customHeight="1">
+      <c r="A60" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D60" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E59" s="7"/>
-      <c r="F59" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="G59" s="8">
+      <c r="E60" s="7"/>
+      <c r="F60" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G60" s="8">
         <v>46287.0</v>
       </c>
-      <c r="H59" s="8">
+      <c r="H60" s="8">
         <v>46295.0</v>
       </c>
-      <c r="I59" s="8"/>
-      <c r="J59" s="9"/>
-      <c r="K59" s="9"/>
-      <c r="L59" s="9"/>
-    </row>
-    <row r="60" ht="29.25" customHeight="1">
-      <c r="A60" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B60" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="C60" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="D60" s="13" t="s">
+      <c r="I60" s="8"/>
+      <c r="J60" s="9"/>
+      <c r="K60" s="9"/>
+      <c r="L60" s="9"/>
+    </row>
+    <row r="61" ht="29.25" customHeight="1">
+      <c r="A61" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B61" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="C61" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D61" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="E60" s="13"/>
-      <c r="F60" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="G60" s="14">
+      <c r="E61" s="13"/>
+      <c r="F61" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G61" s="14">
         <v>46287.0</v>
       </c>
-      <c r="H60" s="14">
+      <c r="H61" s="14">
         <v>46293.0</v>
       </c>
-      <c r="I60" s="14"/>
-      <c r="J60" s="15"/>
-      <c r="K60" s="15"/>
-      <c r="L60" s="15"/>
-      <c r="M60" s="16"/>
-      <c r="N60" s="16"/>
-      <c r="O60" s="16"/>
-      <c r="P60" s="16"/>
-      <c r="Q60" s="16"/>
-      <c r="R60" s="16"/>
-      <c r="S60" s="16"/>
-      <c r="T60" s="16"/>
-      <c r="U60" s="16"/>
-      <c r="V60" s="16"/>
-      <c r="W60" s="16"/>
-      <c r="X60" s="16"/>
-      <c r="Y60" s="16"/>
-      <c r="Z60" s="16"/>
-      <c r="AA60" s="16"/>
-      <c r="AB60" s="16"/>
-      <c r="AC60" s="16"/>
-      <c r="AD60" s="16"/>
-      <c r="AE60" s="16"/>
-    </row>
-    <row r="61" ht="29.25" customHeight="1">
-      <c r="A61" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B61" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="C61" s="6" t="s">
+      <c r="I61" s="14"/>
+      <c r="J61" s="15"/>
+      <c r="K61" s="15"/>
+      <c r="L61" s="15"/>
+      <c r="M61" s="16"/>
+      <c r="N61" s="16"/>
+      <c r="O61" s="16"/>
+      <c r="P61" s="16"/>
+      <c r="Q61" s="16"/>
+      <c r="R61" s="16"/>
+      <c r="S61" s="16"/>
+      <c r="T61" s="16"/>
+      <c r="U61" s="16"/>
+      <c r="V61" s="16"/>
+      <c r="W61" s="16"/>
+      <c r="X61" s="16"/>
+      <c r="Y61" s="16"/>
+      <c r="Z61" s="16"/>
+      <c r="AA61" s="16"/>
+      <c r="AB61" s="16"/>
+      <c r="AC61" s="16"/>
+      <c r="AD61" s="16"/>
+      <c r="AE61" s="16"/>
+    </row>
+    <row r="62" ht="29.25" customHeight="1">
+      <c r="A62" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B62" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="D61" s="7" t="s">
+      <c r="C62" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D62" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E61" s="7"/>
-      <c r="F61" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="G61" s="8">
+      <c r="E62" s="7"/>
+      <c r="F62" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G62" s="8">
         <v>46296.0</v>
       </c>
-      <c r="H61" s="8">
+      <c r="H62" s="8">
         <v>46303.0</v>
       </c>
-      <c r="I61" s="8"/>
-      <c r="J61" s="9"/>
-      <c r="K61" s="9"/>
-      <c r="L61" s="9"/>
-    </row>
-    <row r="62" ht="29.25" customHeight="1">
-      <c r="A62" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="B62" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="C62" s="12" t="s">
+      <c r="I62" s="8"/>
+      <c r="J62" s="9"/>
+      <c r="K62" s="9"/>
+      <c r="L62" s="9"/>
+    </row>
+    <row r="63" ht="29.25" customHeight="1">
+      <c r="A63" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="B63" s="11" t="s">
         <v>102</v>
       </c>
-      <c r="D62" s="13"/>
-      <c r="E62" s="13"/>
-      <c r="F62" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="G62" s="14">
+      <c r="C63" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D63" s="13"/>
+      <c r="E63" s="13"/>
+      <c r="F63" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="G63" s="14">
         <v>46303.0</v>
       </c>
-      <c r="H62" s="14">
+      <c r="H63" s="14">
         <v>46303.0</v>
       </c>
-      <c r="I62" s="14"/>
-      <c r="J62" s="15"/>
-      <c r="K62" s="15"/>
-      <c r="L62" s="15"/>
-      <c r="M62" s="16"/>
-      <c r="N62" s="16"/>
-      <c r="O62" s="16"/>
-      <c r="P62" s="16"/>
-      <c r="Q62" s="16"/>
-      <c r="R62" s="16"/>
-      <c r="S62" s="16"/>
-      <c r="T62" s="16"/>
-      <c r="U62" s="16"/>
-      <c r="V62" s="16"/>
-      <c r="W62" s="16"/>
-      <c r="X62" s="16"/>
-      <c r="Y62" s="16"/>
-      <c r="Z62" s="16"/>
-      <c r="AA62" s="16"/>
-      <c r="AB62" s="16"/>
-      <c r="AC62" s="16"/>
-      <c r="AD62" s="16"/>
-      <c r="AE62" s="16"/>
-    </row>
-    <row r="63" ht="29.25" customHeight="1">
-      <c r="A63" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B63" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="C63" s="6" t="s">
+      <c r="I63" s="14"/>
+      <c r="J63" s="15"/>
+      <c r="K63" s="15"/>
+      <c r="L63" s="15"/>
+      <c r="M63" s="16"/>
+      <c r="N63" s="16"/>
+      <c r="O63" s="16"/>
+      <c r="P63" s="16"/>
+      <c r="Q63" s="16"/>
+      <c r="R63" s="16"/>
+      <c r="S63" s="16"/>
+      <c r="T63" s="16"/>
+      <c r="U63" s="16"/>
+      <c r="V63" s="16"/>
+      <c r="W63" s="16"/>
+      <c r="X63" s="16"/>
+      <c r="Y63" s="16"/>
+      <c r="Z63" s="16"/>
+      <c r="AA63" s="16"/>
+      <c r="AB63" s="16"/>
+      <c r="AC63" s="16"/>
+      <c r="AD63" s="16"/>
+      <c r="AE63" s="16"/>
+    </row>
+    <row r="64" ht="29.25" customHeight="1">
+      <c r="A64" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D63" s="7" t="s">
+      <c r="C64" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D64" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="E63" s="7"/>
-      <c r="F63" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="G63" s="8">
+      <c r="E64" s="7"/>
+      <c r="F64" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="G64" s="8">
         <v>46305.0</v>
       </c>
-      <c r="H63" s="8">
+      <c r="H64" s="8">
         <v>46305.0</v>
       </c>
-      <c r="I63" s="8"/>
-      <c r="J63" s="9"/>
-      <c r="K63" s="9"/>
-      <c r="L63" s="9"/>
-    </row>
-    <row r="64" ht="29.25" customHeight="1">
-      <c r="A64" s="23"/>
-      <c r="B64" s="6"/>
-      <c r="C64" s="24"/>
-      <c r="D64" s="25"/>
-      <c r="E64" s="21"/>
-      <c r="F64" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="G64" s="27"/>
-      <c r="H64" s="27"/>
-      <c r="I64" s="27"/>
-      <c r="J64" s="17"/>
-      <c r="K64" s="21"/>
-      <c r="L64" s="21"/>
+      <c r="I64" s="8"/>
+      <c r="J64" s="9"/>
+      <c r="K64" s="9"/>
+      <c r="L64" s="9"/>
     </row>
     <row r="65" ht="29.25" customHeight="1">
       <c r="A65" s="23"/>
@@ -3467,20 +3503,22 @@
     <row r="69" ht="29.25" customHeight="1">
       <c r="A69" s="23"/>
       <c r="B69" s="6"/>
-      <c r="C69" s="28"/>
+      <c r="C69" s="24"/>
       <c r="D69" s="25"/>
-      <c r="E69" s="29"/>
+      <c r="E69" s="21"/>
       <c r="F69" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="G69" s="30"/>
-      <c r="H69" s="30"/>
-      <c r="I69" s="30"/>
+      <c r="G69" s="27"/>
+      <c r="H69" s="27"/>
+      <c r="I69" s="27"/>
       <c r="J69" s="17"/>
+      <c r="K69" s="21"/>
+      <c r="L69" s="21"/>
     </row>
     <row r="70" ht="29.25" customHeight="1">
-      <c r="A70" s="31"/>
-      <c r="B70" s="28"/>
+      <c r="A70" s="23"/>
+      <c r="B70" s="6"/>
       <c r="C70" s="28"/>
       <c r="D70" s="25"/>
       <c r="E70" s="29"/>
@@ -4456,7 +4494,7 @@
       <c r="G139" s="30"/>
       <c r="H139" s="30"/>
       <c r="I139" s="30"/>
-      <c r="J139" s="32"/>
+      <c r="J139" s="17"/>
     </row>
     <row r="140" ht="29.25" customHeight="1">
       <c r="A140" s="31"/>
@@ -9320,7 +9358,11 @@
       <c r="A487" s="31"/>
       <c r="B487" s="28"/>
       <c r="C487" s="28"/>
+      <c r="D487" s="25"/>
       <c r="E487" s="29"/>
+      <c r="F487" s="26" t="s">
+        <v>69</v>
+      </c>
       <c r="G487" s="30"/>
       <c r="H487" s="30"/>
       <c r="I487" s="30"/>
@@ -14886,50 +14928,60 @@
       <c r="I1043" s="30"/>
       <c r="J1043" s="32"/>
     </row>
+    <row r="1044" ht="29.25" customHeight="1">
+      <c r="A1044" s="31"/>
+      <c r="B1044" s="28"/>
+      <c r="C1044" s="28"/>
+      <c r="E1044" s="29"/>
+      <c r="G1044" s="30"/>
+      <c r="H1044" s="30"/>
+      <c r="I1044" s="30"/>
+      <c r="J1044" s="32"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D63">
+  <conditionalFormatting sqref="D2:D64">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Finalizada">
       <formula>NOT(ISERROR(SEARCH(("Finalizada"),(D2))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D63">
+  <conditionalFormatting sqref="D2:D64">
     <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="En Proceso">
       <formula>NOT(ISERROR(SEARCH(("En Proceso"),(D2))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D63">
+  <conditionalFormatting sqref="D2:D64">
     <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="Pendiente de Revision">
       <formula>NOT(ISERROR(SEARCH(("Pendiente de Revision"),(D2))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J1043">
+  <conditionalFormatting sqref="J2:J1044">
     <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="SI">
       <formula>NOT(ISERROR(SEARCH(("SI"),(J2))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E1043">
+  <conditionalFormatting sqref="E2:E1044">
     <cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="Validado">
       <formula>NOT(ISERROR(SEARCH(("Validado"),(E2))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E1043">
+  <conditionalFormatting sqref="E2:E1044">
     <cfRule type="containsText" dxfId="4" priority="6" operator="containsText" text="Revision">
       <formula>NOT(ISERROR(SEARCH(("Revision"),(E2))))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E88">
+  <conditionalFormatting sqref="E2:E89">
     <cfRule type="containsText" dxfId="5" priority="7" operator="containsText" text="Reasignado">
       <formula>NOT(ISERROR(SEARCH(("Reasignado"),(E2))))</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D486">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="D2:D487">
       <formula1>"Sin Comenzar,En Proceso,Finalizada"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E1043">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E2:E1044">
       <formula1>"_,Esperando Revision,En Revision,Reasignado,Validado"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F486">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="F2:F487">
       <formula1>"_,Ignacio,Lucia,Luciano,Gabriel,Lucía"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>